<commit_message>
chore: update schedule tracker with architecture review changes
</commit_message>
<xml_diff>
--- a/WICFL-microsite-schedule.xlsx
+++ b/WICFL-microsite-schedule.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Legend and Assumptions" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Schedule!$A$5:$I$83</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Schedule!$A$5:$I$84</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="271">
   <si>
     <t xml:space="preserve">WICFL Microsite Project - Activity Schedule</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">Build the factory first. Two separate gates: technical repeatability (Gate A) and commercial validation (Gate B).</t>
   </si>
   <si>
-    <t xml:space="preserve">Prepared by Victor  |  Version 1.1  |  25 Aug 2026  |  Pavel research integrated</t>
+    <t xml:space="preserve">Prepared by Victor  |  Version 1.2  |  26 Aug 2026  |  Architecture review applied</t>
   </si>
   <si>
     <t xml:space="preserve">Phase</t>
@@ -153,6 +153,15 @@
     <t xml:space="preserve">W-009. The Phase 3 start date is unconfirmed until this closes</t>
   </si>
   <si>
+    <t xml:space="preserve">0.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm which CRM WICFL uses: same HighLevel instance as WAGS, a sub-account, or something else</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W-096. Blocks 2.5. Surfaced by architecture review, never named before</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.10</t>
   </si>
   <si>
@@ -303,7 +312,7 @@
     <t xml:space="preserve">W-019. Duration adjusts once 0.9 closes. Preferred fix if the ramp runs long is extending this, not compressing Phase 3</t>
   </si>
   <si>
-    <t xml:space="preserve">PHASE 2  |  Framework Build  |  8 Sep - 18 Sep 2026  |  Owner: Victor, with Pavel shadowing</t>
+    <t xml:space="preserve">PHASE 2  |  Framework Build  |  8 Sep - 18 Sep 2026  |  BLOCK A gated by the handoff; BLOCK B gated by the 9 Oct launch</t>
   </si>
   <si>
     <t xml:space="preserve">Phase 2</t>
@@ -336,22 +345,28 @@
     <t xml:space="preserve">Built in from day one, not retrofitted</t>
   </si>
   <si>
+    <t xml:space="preserve">Phase 2 B</t>
+  </si>
+  <si>
     <t xml:space="preserve">2.4</t>
   </si>
   <si>
-    <t xml:space="preserve">Technical SEO baseline: sitemap, robots, canonical, schema.org markup</t>
+    <t xml:space="preserve">[BLOCK B, due 9 Oct] Technical SEO baseline: sitemap, robots, canonical, schema.org markup</t>
   </si>
   <si>
     <t xml:space="preserve">2.5</t>
   </si>
   <si>
-    <t xml:space="preserve">Wire analytics and lead capture, end to end</t>
+    <t xml:space="preserve">[BLOCK B, due 9 Oct] Wire analytics and lead capture, end to end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depends on 0.11, the CRM is undecided</t>
   </si>
   <si>
     <t xml:space="preserve">2.6</t>
   </si>
   <si>
-    <t xml:space="preserve">Tracking phone number as a config value, routed into GoTo</t>
+    <t xml:space="preserve">[BLOCK B, due 9 Oct] Tracking phone number as a config value, routed into GoTo</t>
   </si>
   <si>
     <t xml:space="preserve">Depends on 0.3</t>
@@ -369,7 +384,7 @@
     <t xml:space="preserve">2.8</t>
   </si>
   <si>
-    <t xml:space="preserve">Build CI content differentiation gate that blocks deploys on cross-site similarity</t>
+    <t xml:space="preserve">[BLOCK B] Build CI content differentiation gate that blocks deploys on cross-site similarity</t>
   </si>
   <si>
     <t xml:space="preserve">Protects the portfolio from doorway risk permanently</t>
@@ -378,7 +393,7 @@
     <t xml:space="preserve">2.9</t>
   </si>
   <si>
-    <t xml:space="preserve">Build the QA and launch checklist: technical, SEO, content, mobile, conversion, tracking, deploy</t>
+    <t xml:space="preserve">[BLOCK B, due 9 Oct] Build the QA and launch checklist: technical, SEO, content, mobile, conversion, tracking, deploy</t>
   </si>
   <si>
     <t xml:space="preserve">Pavel + Victor</t>
@@ -546,19 +561,19 @@
     <t xml:space="preserve">6.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Pavel generates and launches Site #3 with no help from Victor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GATE A</t>
+    <t xml:space="preserve">Pavel picks the niche, then generates and launches Site #3 with no help from Victor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GATE A. Content is prepared beforehand and does not count against factory time</t>
   </si>
   <si>
     <t xml:space="preserve">6.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Measure elapsed time against Site #1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pass: 5 working days or fewer AND zero code written by Victor. Fail: return to Phase 5</t>
+    <t xml:space="preserve">Measure factory time and total elapsed time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASS: factory time &lt;=2 working days from approved content + filled config to live QA-passed site, AND zero code by Victor. Elapsed time is informational only</t>
   </si>
   <si>
     <t xml:space="preserve">PHASE 7  |  Provisioning Automation  |  16 Nov - 11 Dec 2026  |  Owner: Victor + Pavel</t>
@@ -609,7 +624,7 @@
     <t xml:space="preserve">Victor moves to advisory only from here</t>
   </si>
   <si>
-    <t xml:space="preserve">PHASE 8  |  SEO Data Window  |  12 Oct 2026 - 5 Feb 2027  |  Runs in parallel. No new sites beyond #3</t>
+    <t xml:space="preserve">PHASE 8  |  SEO Data Window  |  12 Oct 2026 - 26 Feb 2027  |  Runs in parallel. No new sites beyond #3</t>
   </si>
   <si>
     <t xml:space="preserve">Phase 8</t>
@@ -630,7 +645,7 @@
     <t xml:space="preserve">Kevin reviews monthly against the Gate B criteria</t>
   </si>
   <si>
-    <t xml:space="preserve">GATE B  |  Commercial Go / No-Go  |  8 Feb - 12 Feb 2027  |  Owner: Kevin</t>
+    <t xml:space="preserve">GATE B  |  Commercial Go / No-Go  |  1 Mar - 5 Mar 2027  |  Owner: Kevin  |  Moved so Site #2 gets its full 120 days</t>
   </si>
   <si>
     <t xml:space="preserve">Gate B</t>
@@ -642,7 +657,7 @@
     <t xml:space="preserve">Review 120-day performance of Sites #1 and #2 against the criteria set in 0.7</t>
   </si>
   <si>
-    <t xml:space="preserve">GATE B</t>
+    <t xml:space="preserve">GATE B. Site #2 launched 30 Oct, its 120 days land 27 Feb</t>
   </si>
   <si>
     <t xml:space="preserve">9.2</t>
@@ -654,7 +669,7 @@
     <t xml:space="preserve">Pass: proceed to Phase 10. Fail: revisit niches or the microsite model itself</t>
   </si>
   <si>
-    <t xml:space="preserve">PHASE 10  |  Scale to First 20 Sites  |  from 16 Feb 2027  |  Conditional on Gate B</t>
+    <t xml:space="preserve">PHASE 10  |  Scale to First 20 Sites  |  from 8 Mar 2027  |  Conditional on Gate B</t>
   </si>
   <si>
     <t xml:space="preserve">Phase 10</t>
@@ -803,10 +818,16 @@
     <t xml:space="preserve">Indicative only. Nothing in Phase 10 begins unless Gate B passes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Risk: Phase 3 start</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not confirmed. Pavel is ramping on HTML/CSS, Astro, Git and Cloudflare in parallel. Activity 0.9 exists to get his real availability. Moving Site #1's launch moves Gate B, because the launch starts the 120 day clock.</t>
+    <t xml:space="preserve">Phase 2 blocks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Block A is gated by the 18 Sep handoff: schema, template, bilingual routing, generator, handoff. Block B is gated by the 9 Oct launch and is built during Phase 3. The CI differentiation gate must exist before the first content publishes, early October.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gate B date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moved from 12 Feb to 1-5 Mar 2027. Site #2 launches 30 Oct and its 120 days land 27 Feb, after the original gate date.</t>
   </si>
   <si>
     <t xml:space="preserve">Rule: AI and content</t>
@@ -1416,7 +1437,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -1762,14 +1783,14 @@
         <v>20</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>46258</v>
+        <v>46260</v>
       </c>
       <c r="F16" s="9" t="n">
         <v>46269</v>
       </c>
       <c r="G16" s="7" t="n">
         <f aca="false">NETWORKDAYS(E16,F16)</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H16" s="10" t="s">
         <v>17</v>
@@ -1778,61 +1799,61 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
+      <c r="C17" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="D17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="9" t="n">
+        <v>46258</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E17,F17)</f>
+        <v>10</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="8" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E18" s="9" t="n">
-        <v>46265</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>46265</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E18,F18)</f>
-        <v>1</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I18" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B19" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="D19" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>49</v>
       </c>
       <c r="E19" s="9" t="n">
         <v>46265</v>
@@ -1847,20 +1868,22 @@
       <c r="H19" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I19" s="8"/>
+      <c r="I19" s="8" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E20" s="9" t="n">
         <v>46265</v>
@@ -1879,65 +1902,63 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E21" s="9" t="n">
         <v>46265</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="G21" s="7" t="n">
         <f aca="false">NETWORKDAYS(E21,F21)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>17</v>
       </c>
       <c r="I21" s="8"/>
     </row>
-    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="E22" s="9" t="n">
         <v>46265</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="G22" s="7" t="n">
         <f aca="false">NETWORKDAYS(E22,F22)</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I22" s="8"/>
+    </row>
+    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>60</v>
@@ -1946,17 +1967,17 @@
         <v>61</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="F23" s="9" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="G23" s="7" t="n">
         <f aca="false">NETWORKDAYS(E23,F23)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H23" s="10" t="s">
         <v>17</v>
@@ -1965,9 +1986,9 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>63</v>
@@ -1976,99 +1997,99 @@
         <v>64</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E24" s="9" t="n">
         <v>46267</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="G24" s="7" t="n">
         <f aca="false">NETWORKDAYS(E24,F24)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I24" s="8"/>
+      <c r="I24" s="8" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>46269</v>
       </c>
       <c r="G25" s="7" t="n">
         <f aca="false">NETWORKDAYS(E25,F25)</f>
+        <v>3</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="8"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>46268</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>46269</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E26,F26)</f>
         <v>2</v>
       </c>
-      <c r="H25" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-    </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B27" s="7" t="s">
+      <c r="H26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I26" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="C27" s="8" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E27" s="9" t="n">
-        <v>46272</v>
-      </c>
-      <c r="F27" s="9" t="n">
-        <v>46272</v>
-      </c>
-      <c r="G27" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E27,F27)</f>
-        <v>1</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I27" s="8" t="s">
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+    </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
-        <v>69</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>73</v>
@@ -2077,13 +2098,13 @@
         <v>74</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="G28" s="7" t="n">
         <f aca="false">NETWORKDAYS(E28,F28)</f>
@@ -2096,9 +2117,9 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>76</v>
@@ -2107,7 +2128,7 @@
         <v>77</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E29" s="9" t="n">
         <v>46273</v>
@@ -2126,52 +2147,52 @@
         <v>78</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-    </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
+      <c r="C30" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="D30" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>46273</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E30,F30)</f>
+        <v>1</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I30" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C31" s="8" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D31" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E31" s="9" t="n">
-        <v>46265</v>
-      </c>
-      <c r="F31" s="9" t="n">
-        <v>46276</v>
-      </c>
-      <c r="G31" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E31,F31)</f>
-        <v>10</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I31" s="8" t="s">
-        <v>83</v>
-      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>84</v>
@@ -2183,10 +2204,10 @@
         <v>40</v>
       </c>
       <c r="E32" s="9" t="n">
-        <v>46272</v>
+        <v>46265</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="G32" s="7" t="n">
         <f aca="false">NETWORKDAYS(E32,F32)</f>
@@ -2199,9 +2220,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>87</v>
@@ -2226,85 +2247,85 @@
         <v>17</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E34" s="9" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="F34" s="9" t="n">
         <v>46283</v>
       </c>
       <c r="G34" s="7" t="n">
         <f aca="false">NETWORKDAYS(E34,F34)</f>
+        <v>10</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>46273</v>
+      </c>
+      <c r="F35" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E35,F35)</f>
         <v>9</v>
       </c>
-      <c r="H34" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I34" s="8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-    </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B36" s="7" t="s">
+      <c r="H35" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I35" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C36" s="8" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D36" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E36" s="9" t="n">
-        <v>46273</v>
-      </c>
-      <c r="F36" s="9" t="n">
-        <v>46275</v>
-      </c>
-      <c r="G36" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E36,F36)</f>
-        <v>3</v>
-      </c>
-      <c r="H36" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I36" s="8" t="s">
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="B37" s="7" t="s">
         <v>97</v>
@@ -2313,26 +2334,28 @@
         <v>98</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="E37" s="9" t="n">
         <v>46273</v>
       </c>
       <c r="F37" s="9" t="n">
-        <v>46279</v>
+        <v>46275</v>
       </c>
       <c r="G37" s="7" t="n">
         <f aca="false">NETWORKDAYS(E37,F37)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H37" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I37" s="8"/>
+      <c r="I37" s="8" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>100</v>
@@ -2341,28 +2364,26 @@
         <v>101</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="E38" s="9" t="n">
-        <v>46275</v>
+        <v>46273</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>46279</v>
       </c>
       <c r="G38" s="7" t="n">
         <f aca="false">NETWORKDAYS(E38,F38)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H38" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I38" s="8" t="s">
-        <v>102</v>
-      </c>
+      <c r="I38" s="8"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B39" s="7" t="s">
         <v>103</v>
@@ -2371,13 +2392,13 @@
         <v>104</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E39" s="9" t="n">
+        <v>46275</v>
+      </c>
+      <c r="F39" s="9" t="n">
         <v>46279</v>
-      </c>
-      <c r="F39" s="9" t="n">
-        <v>46281</v>
       </c>
       <c r="G39" s="7" t="n">
         <f aca="false">NETWORKDAYS(E39,F39)</f>
@@ -2386,20 +2407,22 @@
       <c r="H39" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I39" s="8"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I39" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="E40" s="9" t="n">
         <v>46279</v>
@@ -2418,206 +2441,206 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="E41" s="9" t="n">
-        <v>46280</v>
+        <v>46293</v>
       </c>
       <c r="F41" s="9" t="n">
-        <v>46281</v>
+        <v>46297</v>
       </c>
       <c r="G41" s="7" t="n">
         <f aca="false">NETWORKDAYS(E41,F41)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H41" s="10" t="s">
         <v>17</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E42" s="9" t="n">
         <v>46280</v>
       </c>
       <c r="F42" s="9" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="G42" s="7" t="n">
         <f aca="false">NETWORKDAYS(E42,F42)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H42" s="10" t="s">
         <v>17</v>
       </c>
       <c r="I42" s="8" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E43" s="9" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="F43" s="9" t="n">
         <v>46282</v>
       </c>
       <c r="G43" s="7" t="n">
         <f aca="false">NETWORKDAYS(E43,F43)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H43" s="10" t="s">
         <v>17</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>118</v>
+        <v>52</v>
       </c>
       <c r="E44" s="9" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="G44" s="7" t="n">
         <f aca="false">NETWORKDAYS(E44,F44)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H44" s="10" t="s">
         <v>17</v>
       </c>
       <c r="I44" s="8" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="E45" s="9" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="F45" s="9" t="n">
         <v>46283</v>
       </c>
       <c r="G45" s="7" t="n">
         <f aca="false">NETWORKDAYS(E45,F45)</f>
+        <v>4</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I45" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>46283</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E46,F46)</f>
         <v>1</v>
       </c>
-      <c r="H45" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I45" s="8" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="B46" s="5"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="5"/>
-      <c r="H46" s="5"/>
-      <c r="I46" s="5"/>
-    </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B47" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E47" s="9" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F47" s="9" t="n">
-        <v>46286</v>
-      </c>
-      <c r="G47" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E47,F47)</f>
-        <v>1</v>
-      </c>
-      <c r="H47" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I47" s="8" t="s">
+      <c r="H46" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I46" s="8" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+      <c r="I47" s="5"/>
+    </row>
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>40</v>
@@ -2626,97 +2649,99 @@
         <v>46286</v>
       </c>
       <c r="F48" s="9" t="n">
-        <v>46290</v>
+        <v>46286</v>
       </c>
       <c r="G48" s="7" t="n">
         <f aca="false">NETWORKDAYS(E48,F48)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H48" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I48" s="8"/>
+      <c r="I48" s="8" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>132</v>
+        <v>40</v>
       </c>
       <c r="E49" s="9" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="F49" s="9" t="n">
-        <v>46301</v>
+        <v>46290</v>
       </c>
       <c r="G49" s="7" t="n">
         <f aca="false">NETWORKDAYS(E49,F49)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H49" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I49" s="8" t="s">
-        <v>133</v>
-      </c>
+      <c r="I49" s="8"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>40</v>
+        <v>137</v>
       </c>
       <c r="E50" s="9" t="n">
-        <v>46300</v>
+        <v>46288</v>
       </c>
       <c r="F50" s="9" t="n">
         <v>46301</v>
       </c>
       <c r="G50" s="7" t="n">
         <f aca="false">NETWORKDAYS(E50,F50)</f>
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H50" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I50" s="8"/>
+      <c r="I50" s="8" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E51" s="9" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F51" s="9" t="n">
         <v>46301</v>
-      </c>
-      <c r="F51" s="9" t="n">
-        <v>46303</v>
       </c>
       <c r="G51" s="7" t="n">
         <f aca="false">NETWORKDAYS(E51,F51)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H51" s="10" t="s">
         <v>17</v>
@@ -2725,26 +2750,26 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E52" s="9" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="F52" s="9" t="n">
         <v>46303</v>
       </c>
       <c r="G52" s="7" t="n">
         <f aca="false">NETWORKDAYS(E52,F52)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H52" s="10" t="s">
         <v>17</v>
@@ -2753,22 +2778,22 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E53" s="9" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="F53" s="9" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="G53" s="7" t="n">
         <f aca="false">NETWORKDAYS(E53,F53)</f>
@@ -2777,19 +2802,17 @@
       <c r="H53" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I53" s="8" t="s">
-        <v>142</v>
-      </c>
+      <c r="I53" s="8"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D54" s="6" t="s">
         <v>40</v>
@@ -2807,60 +2830,60 @@
       <c r="H54" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I54" s="8"/>
-    </row>
-    <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="B56" s="7" t="s">
+      <c r="I54" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="C56" s="8" t="s">
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B55" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="D56" s="6" t="s">
+      <c r="C55" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E56" s="9" t="n">
-        <v>46307</v>
-      </c>
-      <c r="F56" s="9" t="n">
-        <v>46307</v>
-      </c>
-      <c r="G56" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E56,F56)</f>
+      <c r="E55" s="9" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>46304</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E55,F55)</f>
         <v>1</v>
       </c>
-      <c r="H56" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I56" s="8" t="s">
-        <v>149</v>
-      </c>
+      <c r="H55" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I55" s="8"/>
+    </row>
+    <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>40</v>
@@ -2869,97 +2892,99 @@
         <v>46307</v>
       </c>
       <c r="F57" s="9" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="G57" s="7" t="n">
         <f aca="false">NETWORKDAYS(E57,F57)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H57" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I57" s="8"/>
+      <c r="I57" s="8" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>154</v>
+        <v>40</v>
       </c>
       <c r="E58" s="9" t="n">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="F58" s="9" t="n">
-        <v>46322</v>
+        <v>46311</v>
       </c>
       <c r="G58" s="7" t="n">
         <f aca="false">NETWORKDAYS(E58,F58)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H58" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I58" s="8" t="s">
-        <v>155</v>
-      </c>
+      <c r="I58" s="8"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>40</v>
+        <v>159</v>
       </c>
       <c r="E59" s="9" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F59" s="9" t="n">
         <v>46322</v>
-      </c>
-      <c r="F59" s="9" t="n">
-        <v>46324</v>
       </c>
       <c r="G59" s="7" t="n">
         <f aca="false">NETWORKDAYS(E59,F59)</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H59" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I59" s="8"/>
+      <c r="I59" s="8" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D60" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E60" s="9" t="n">
-        <v>46325</v>
+        <v>46322</v>
       </c>
       <c r="F60" s="9" t="n">
-        <v>46325</v>
+        <v>46324</v>
       </c>
       <c r="G60" s="7" t="n">
         <f aca="false">NETWORKDAYS(E60,F60)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H60" s="10" t="s">
         <v>17</v>
@@ -2968,13 +2993,13 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>40</v>
@@ -2994,69 +3019,69 @@
       </c>
       <c r="I61" s="8"/>
     </row>
-    <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="B62" s="5"/>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-      <c r="G62" s="5"/>
-      <c r="H62" s="5"/>
-      <c r="I62" s="5"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="B63" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="C63" s="8" t="s">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B62" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="D63" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E63" s="9" t="n">
-        <v>46328</v>
-      </c>
-      <c r="F63" s="9" t="n">
-        <v>46329</v>
-      </c>
-      <c r="G63" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E63,F63)</f>
-        <v>2</v>
-      </c>
-      <c r="H63" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I63" s="8"/>
+      <c r="C62" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F62" s="9" t="n">
+        <v>46325</v>
+      </c>
+      <c r="G62" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E62,F62)</f>
+        <v>1</v>
+      </c>
+      <c r="H62" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I62" s="8"/>
+    </row>
+    <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="B63" s="5"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+      <c r="I63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E64" s="9" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F64" s="9" t="n">
         <v>46329</v>
-      </c>
-      <c r="F64" s="9" t="n">
-        <v>46331</v>
       </c>
       <c r="G64" s="7" t="n">
         <f aca="false">NETWORKDAYS(E64,F64)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H64" s="10" t="s">
         <v>17</v>
@@ -3065,198 +3090,198 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="E65" s="9" t="n">
+        <v>46329</v>
+      </c>
+      <c r="F65" s="9" t="n">
         <v>46331</v>
-      </c>
-      <c r="F65" s="9" t="n">
-        <v>46332</v>
       </c>
       <c r="G65" s="7" t="n">
         <f aca="false">NETWORKDAYS(E65,F65)</f>
+        <v>3</v>
+      </c>
+      <c r="H65" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I65" s="8"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B66" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>46331</v>
+      </c>
+      <c r="F66" s="9" t="n">
+        <v>46332</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E66,F66)</f>
         <v>2</v>
       </c>
-      <c r="H65" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I65" s="8"/>
-    </row>
-    <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="B66" s="11"/>
-      <c r="C66" s="11"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="11"/>
-      <c r="F66" s="11"/>
-      <c r="G66" s="11"/>
-      <c r="H66" s="11"/>
-      <c r="I66" s="11"/>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="B67" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C67" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="D67" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="E67" s="15" t="n">
-        <v>46335</v>
-      </c>
-      <c r="F67" s="15" t="n">
-        <v>46339</v>
-      </c>
-      <c r="G67" s="13" t="n">
-        <f aca="false">NETWORKDAYS(E67,F67)</f>
-        <v>5</v>
-      </c>
-      <c r="H67" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="I67" s="14" t="s">
-        <v>174</v>
-      </c>
+      <c r="H66" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I66" s="8"/>
+    </row>
+    <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="B67" s="11"/>
+      <c r="C67" s="11"/>
+      <c r="D67" s="11"/>
+      <c r="E67" s="11"/>
+      <c r="F67" s="11"/>
+      <c r="G67" s="11"/>
+      <c r="H67" s="11"/>
+      <c r="I67" s="11"/>
     </row>
     <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="12" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D68" s="12" t="s">
         <v>40</v>
       </c>
       <c r="E68" s="15" t="n">
-        <v>46339</v>
+        <v>46335</v>
       </c>
       <c r="F68" s="15" t="n">
         <v>46339</v>
       </c>
       <c r="G68" s="13" t="n">
         <f aca="false">NETWORKDAYS(E68,F68)</f>
+        <v>5</v>
+      </c>
+      <c r="H68" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="I68" s="14" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="B69" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="C69" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E69" s="15" t="n">
+        <v>46339</v>
+      </c>
+      <c r="F69" s="15" t="n">
+        <v>46339</v>
+      </c>
+      <c r="G69" s="13" t="n">
+        <f aca="false">NETWORKDAYS(E69,F69)</f>
         <v>1</v>
       </c>
-      <c r="H68" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="I68" s="14" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="B69" s="5"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
-      <c r="G69" s="5"/>
-      <c r="H69" s="5"/>
-      <c r="I69" s="5"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="B70" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C70" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="D70" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E70" s="9" t="n">
-        <v>46342</v>
-      </c>
-      <c r="F70" s="9" t="n">
-        <v>46346</v>
-      </c>
-      <c r="G70" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E70,F70)</f>
-        <v>5</v>
-      </c>
-      <c r="H70" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I70" s="8" t="s">
+      <c r="H69" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="I69" s="14" t="s">
         <v>182</v>
       </c>
+    </row>
+    <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B70" s="5"/>
+      <c r="C70" s="5"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="5"/>
+      <c r="I70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E71" s="9" t="n">
+        <v>46342</v>
+      </c>
+      <c r="F71" s="9" t="n">
         <v>46346</v>
-      </c>
-      <c r="F71" s="9" t="n">
-        <v>46353</v>
       </c>
       <c r="G71" s="7" t="n">
         <f aca="false">NETWORKDAYS(E71,F71)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H71" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I71" s="8"/>
+      <c r="I71" s="8" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E72" s="9" t="n">
-        <v>46356</v>
+        <v>46346</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>46360</v>
+        <v>46353</v>
       </c>
       <c r="G72" s="7" t="n">
         <f aca="false">NETWORKDAYS(E72,F72)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H72" s="10" t="s">
         <v>17</v>
@@ -3265,26 +3290,26 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E73" s="9" t="n">
-        <v>46358</v>
+        <v>46356</v>
       </c>
       <c r="F73" s="9" t="n">
         <v>46360</v>
       </c>
       <c r="G73" s="7" t="n">
         <f aca="false">NETWORKDAYS(E73,F73)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H73" s="10" t="s">
         <v>17</v>
@@ -3293,26 +3318,26 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E74" s="9" t="n">
-        <v>46363</v>
+        <v>46358</v>
       </c>
       <c r="F74" s="9" t="n">
-        <v>46366</v>
+        <v>46360</v>
       </c>
       <c r="G74" s="7" t="n">
         <f aca="false">NETWORKDAYS(E74,F74)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H74" s="10" t="s">
         <v>17</v>
@@ -3321,237 +3346,265 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="E75" s="9" t="n">
-        <v>46367</v>
+        <v>46363</v>
       </c>
       <c r="F75" s="9" t="n">
-        <v>46367</v>
+        <v>46366</v>
       </c>
       <c r="G75" s="7" t="n">
         <f aca="false">NETWORKDAYS(E75,F75)</f>
+        <v>4</v>
+      </c>
+      <c r="H75" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I75" s="8"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>46367</v>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>46367</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E76,F76)</f>
         <v>1</v>
       </c>
-      <c r="H75" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I75" s="8" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B76" s="5"/>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
-      <c r="G76" s="5"/>
-      <c r="H76" s="5"/>
-      <c r="I76" s="5"/>
-    </row>
-    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="B77" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="C77" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="D77" s="6" t="s">
+      <c r="H76" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I76" s="8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="B77" s="5"/>
+      <c r="C77" s="5"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="5"/>
+      <c r="H77" s="5"/>
+      <c r="I77" s="5"/>
+    </row>
+    <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B78" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="D78" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E77" s="9" t="n">
+      <c r="E78" s="9" t="n">
         <v>46307</v>
       </c>
-      <c r="F77" s="9" t="n">
-        <v>46423</v>
-      </c>
-      <c r="G77" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E77,F77)</f>
-        <v>85</v>
-      </c>
-      <c r="H77" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I77" s="8" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="B78" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="C78" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="D78" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E78" s="9" t="n">
-        <v>46328</v>
-      </c>
       <c r="F78" s="9" t="n">
-        <v>46423</v>
+        <v>46444</v>
       </c>
       <c r="G78" s="7" t="n">
         <f aca="false">NETWORKDAYS(E78,F78)</f>
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="H78" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="I78" s="8"/>
-    </row>
-    <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="B79" s="11"/>
-      <c r="C79" s="11"/>
-      <c r="D79" s="11"/>
-      <c r="E79" s="11"/>
-      <c r="F79" s="11"/>
-      <c r="G79" s="11"/>
-      <c r="H79" s="11"/>
-      <c r="I79" s="11"/>
-    </row>
-    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="B80" s="13" t="s">
+      <c r="I78" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="C80" s="14" t="s">
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B79" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="D80" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="E80" s="15" t="n">
-        <v>46426</v>
-      </c>
-      <c r="F80" s="15" t="n">
-        <v>46429</v>
-      </c>
-      <c r="G80" s="13" t="n">
-        <f aca="false">NETWORKDAYS(E80,F80)</f>
-        <v>4</v>
-      </c>
-      <c r="H80" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="I80" s="14" t="s">
+      <c r="C79" s="8" t="s">
         <v>205</v>
       </c>
+      <c r="D79" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E79" s="9" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F79" s="9" t="n">
+        <v>46444</v>
+      </c>
+      <c r="G79" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E79,F79)</f>
+        <v>85</v>
+      </c>
+      <c r="H79" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I79" s="8"/>
+    </row>
+    <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="B80" s="11"/>
+      <c r="C80" s="11"/>
+      <c r="D80" s="11"/>
+      <c r="E80" s="11"/>
+      <c r="F80" s="11"/>
+      <c r="G80" s="11"/>
+      <c r="H80" s="11"/>
+      <c r="I80" s="11"/>
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D81" s="12" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="E81" s="15" t="n">
-        <v>46430</v>
+        <v>46447</v>
       </c>
       <c r="F81" s="15" t="n">
-        <v>46430</v>
+        <v>46450</v>
       </c>
       <c r="G81" s="13" t="n">
         <f aca="false">NETWORKDAYS(E81,F81)</f>
+        <v>4</v>
+      </c>
+      <c r="H81" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="I81" s="14" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="B82" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="C82" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="D82" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E82" s="15" t="n">
+        <v>46451</v>
+      </c>
+      <c r="F82" s="15" t="n">
+        <v>46451</v>
+      </c>
+      <c r="G82" s="13" t="n">
+        <f aca="false">NETWORKDAYS(E82,F82)</f>
         <v>1</v>
       </c>
-      <c r="H81" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="I81" s="14" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="B82" s="5"/>
-      <c r="C82" s="5"/>
-      <c r="D82" s="5"/>
-      <c r="E82" s="5"/>
-      <c r="F82" s="5"/>
-      <c r="G82" s="5"/>
-      <c r="H82" s="5"/>
-      <c r="I82" s="5"/>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="B83" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="C83" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="D83" s="6" t="s">
+      <c r="H82" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="I82" s="14" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="B83" s="5"/>
+      <c r="C83" s="5"/>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="5"/>
+      <c r="G83" s="5"/>
+      <c r="H83" s="5"/>
+      <c r="I83" s="5"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="B84" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="D84" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E83" s="9" t="n">
-        <v>46434</v>
-      </c>
-      <c r="F83" s="9" t="n">
-        <v>46507</v>
-      </c>
-      <c r="G83" s="7" t="n">
-        <f aca="false">NETWORKDAYS(E83,F83)</f>
-        <v>54</v>
-      </c>
-      <c r="H83" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I83" s="8" t="s">
-        <v>213</v>
+      <c r="E84" s="9" t="n">
+        <v>46454</v>
+      </c>
+      <c r="F84" s="9" t="n">
+        <v>46528</v>
+      </c>
+      <c r="G84" s="7" t="n">
+        <f aca="false">NETWORKDAYS(E84,F84)</f>
+        <v>55</v>
+      </c>
+      <c r="H84" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="I84" s="8" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I83"/>
+  <autoFilter ref="A5:I84"/>
   <mergeCells count="13">
     <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A46:I46"/>
-    <mergeCell ref="A55:I55"/>
-    <mergeCell ref="A62:I62"/>
-    <mergeCell ref="A66:I66"/>
-    <mergeCell ref="A69:I69"/>
-    <mergeCell ref="A76:I76"/>
-    <mergeCell ref="A79:I79"/>
-    <mergeCell ref="A82:I82"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A63:I63"/>
+    <mergeCell ref="A67:I67"/>
+    <mergeCell ref="A70:I70"/>
+    <mergeCell ref="A77:I77"/>
+    <mergeCell ref="A80:I80"/>
+    <mergeCell ref="A83:I83"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3580,40 +3633,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C5" s="18" t="n">
         <v>46339</v>
@@ -3622,18 +3675,18 @@
         <v>40</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="C6" s="18" t="n">
         <v>46430</v>
@@ -3642,20 +3695,20 @@
         <v>20</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="19" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="20"/>
@@ -3682,7 +3735,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -3691,71 +3744,71 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3764,70 +3817,78 @@
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="22" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="22" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23"/>
-      <c r="B19" s="24"/>
-    </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="s">
-        <v>262</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>263</v>
+        <v>266</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="22" t="s">
+        <v>267</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="23"/>
+      <c r="B20" s="24"/>
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="22" t="s">
+        <v>269</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>